<commit_message>
Publish VitalSigns/TestBuild to publish-master bb37c339d873cd6cfa8d520a698bbb0b86a024cd
</commit_message>
<xml_diff>
--- a/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
+++ b/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.0</t>
+    <t>0.9.74</t>
   </si>
   <si>
     <t>Name</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Confounding factor is Issues or factors that may impact on &lt;the measurement&gt;, not captured in other fields</t>
+    <t>Confounding factor is for comments on and records of other incidental factors that may be affect interpretation of the observation, not captured in other fields</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
Publish VitalSigns/NordicTXTestBuild to publish-master f9bbb8e27129ca78fa0142749bac59a4acaeffb5
</commit_message>
<xml_diff>
--- a/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
+++ b/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.74</t>
+    <t>0.9.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Confounding factor is for comments on and records of other incidental factors that may be affect interpretation of the observation, not captured in other fields</t>
+    <t>Confounding factor is Issues or factors that may impact on &lt;the measurement&gt;, not captured in other fields</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
Publish VitalSigns/TestBuild to publish-master f9bbb8e27129ca78fa0142749bac59a4acaeffb5
</commit_message>
<xml_diff>
--- a/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
+++ b/publish/StructureDefinition-NoDomainVitalSignsConfoundingFactorExtension.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.2</t>
+    <t>0.9.74</t>
   </si>
   <si>
     <t>Name</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Confounding factor is Issues or factors that may impact on &lt;the measurement&gt;, not captured in other fields</t>
+    <t>Confounding factor is for comments on and records of other incidental factors that may be affect interpretation of the observation, not captured in other fields</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>